<commit_message>
test: verify diagnostic aggregation and add struct-mismatch test
Reviewer of c4 noted two gaps:
- bad_int_range.xlsx had 1 out-of-range cell; new aggregation spec
  needs >= 2 to prove the collect-don't-fail-fast behavior
- bad_struct_field.xlsx existed but had no test

Both addressed. Aggregation test now asserts errs.len() >= 2 of
ValueOutOfRange; struct test asserts StructField(Mismatch|CountMismatch).
</commit_message>
<xml_diff>
--- a/tablec-core/tests/fixtures/error_cases/bad_int_range.xlsx
+++ b/tablec-core/tests/fixtures/error_cases/bad_int_range.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:1">
@@ -374,6 +374,11 @@
         <v>200</v>
       </c>
     </row>
+    <row r="7" spans="1:1">
+      <c r="A7">
+        <v>300</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>